<commit_message>
[ROT] Add standalone loader for programming scripts
</commit_message>
<xml_diff>
--- a/Projects/NUCLEO-H563ZI/ROT_Provisioning/OEMiROT_OEMuROT/OEMiROT_OEMuROT_flash_layout.xlsx
+++ b/Projects/NUCLEO-H563ZI/ROT_Provisioning/OEMiROT_OEMuROT/OEMiROT_OEMuROT_flash_layout.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ST\Cube\Cube1\STM32CubeH5\Projects\NUCLEO-H563ZI\ROT_Provisioning\OEMiROT_OEMuROT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{838F360E-8C81-4281-B10E-EF18D625C36C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EDE1516-6446-431D-9E95-0DDAD7C68D3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28965" yWindow="-165" windowWidth="29130" windowHeight="15810" xr2:uid="{973ADE99-8809-4282-875C-44A8EA15E93C}"/>
   </bookViews>
   <sheets>
     <sheet name="OEMiROT+OEMuROT Flash Layout" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -63,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="40">
   <si>
     <t>offset</t>
   </si>
@@ -101,12 +102,6 @@
     <t>Y</t>
   </si>
   <si>
-    <t>App Active</t>
-  </si>
-  <si>
-    <t>App Download</t>
-  </si>
-  <si>
     <t>Data Active</t>
   </si>
   <si>
@@ -186,6 +181,9 @@
   </si>
   <si>
     <t>OEMUROT (Download)</t>
+  </si>
+  <si>
+    <t>App not in max size</t>
   </si>
 </sst>
 </file>
@@ -224,7 +222,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="3" tint="0.89999084444715716"/>
+        <fgColor theme="9" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -256,7 +254,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -295,6 +293,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -709,7 +710,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5EEE003-AB81-416D-8FF7-83C8B34AB91C}">
-  <dimension ref="A1:L38"/>
+  <dimension ref="A1:L40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.42578125" bestFit="1" customWidth="1"/>
@@ -743,7 +744,7 @@
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B4" s="6">
         <v>200000</v>
@@ -751,7 +752,7 @@
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B5" s="6">
         <v>2000</v>
@@ -773,7 +774,7 @@
         <v>11</v>
       </c>
       <c r="C7" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
@@ -784,21 +785,21 @@
         <v>11</v>
       </c>
       <c r="C8" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B9" s="1">
-        <f>IF(($B$8="Y"),8000,0)</f>
-        <v>8000</v>
+        <f>IF(($B$8="Y"),6000,0)</f>
+        <v>6000</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>6</v>
@@ -806,14 +807,14 @@
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B11" s="4">
         <f>IF(($B$10="Y"),$B$5,0)</f>
         <v>0</v>
       </c>
       <c r="C11" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
@@ -821,7 +822,7 @@
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B13" s="7" t="s">
         <v>3</v>
@@ -833,31 +834,31 @@
         <v>1</v>
       </c>
       <c r="E13" s="7" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G13" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="H13" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I13" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="J13" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="H13" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="I13" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="J13" s="12" t="s">
-        <v>28</v>
-      </c>
       <c r="K13" s="12" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="L13" s="6"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>2</v>
@@ -870,8 +871,8 @@
         <v>8000000</v>
       </c>
       <c r="E14" s="3" t="str">
-        <f>DEC2HEX(HEX2DEC(D14)+HEX2DEC(F14)-1)</f>
-        <v>8017FFF</v>
+        <f>DEC2HEX(HEX2DEC(D14)+IF(($B$8="Y"),HEX2DEC(F14)-HEX2DEC(F15),HEX2DEC(F14))-1)</f>
+        <v>8011FFF</v>
       </c>
       <c r="F14" s="8">
         <v>18000</v>
@@ -898,67 +899,67 @@
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="B15" s="3">
-        <v>0</v>
+        <v>10</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>10</v>
       </c>
       <c r="C15" s="3" t="str">
+        <f>DEC2HEX(HEX2DEC(C14)+HEX2DEC(F14)-HEX2DEC(F15))</f>
+        <v>12000</v>
+      </c>
+      <c r="D15" s="3" t="str">
+        <f>DEC2HEX(HEX2DEC($B$3)+HEX2DEC(C15))</f>
+        <v>8012000</v>
+      </c>
+      <c r="E15" s="3" t="str">
+        <f>DEC2HEX(HEX2DEC(D15)+HEX2DEC(F15)-1)</f>
+        <v>8017FFF</v>
+      </c>
+      <c r="F15" s="8">
+        <f>$B$9</f>
+        <v>6000</v>
+      </c>
+      <c r="G15" s="3">
+        <f>H15/1024</f>
+        <v>24</v>
+      </c>
+      <c r="H15" s="2">
+        <f>HEX2DEC(F15)</f>
+        <v>24576</v>
+      </c>
+      <c r="I15" s="13">
+        <f>H15/HEX2DEC($B$5)</f>
+        <v>3</v>
+      </c>
+      <c r="J15" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="K15" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="L15" s="4"/>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A16" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="B16" s="3">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="str">
         <f>DEC2HEX(HEX2DEC(C14)+HEX2DEC(F14))</f>
         <v>18000</v>
       </c>
-      <c r="D15" s="3" t="str">
-        <f>DEC2HEX(HEX2DEC($B$3)+HEX2DEC(C15))</f>
+      <c r="D16" s="3" t="str">
+        <f>DEC2HEX(HEX2DEC($B$3)+HEX2DEC(C16))</f>
         <v>8018000</v>
-      </c>
-      <c r="E15" s="3" t="str">
-        <f>DEC2HEX(HEX2DEC(D15)+HEX2DEC(F15)-1)</f>
-        <v>8029FFF</v>
-      </c>
-      <c r="F15" s="8">
-        <v>12000</v>
-      </c>
-      <c r="G15" s="3">
-        <f>H15/1024</f>
-        <v>72</v>
-      </c>
-      <c r="H15" s="2">
-        <f>HEX2DEC(F15)</f>
-        <v>73728</v>
-      </c>
-      <c r="I15" s="13">
-        <f>H15/HEX2DEC($B$5)</f>
-        <v>9</v>
-      </c>
-      <c r="J15" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="K15" s="13" t="s">
-        <v>6</v>
-      </c>
-      <c r="L15" s="4"/>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A16" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="B16" s="3">
-        <v>2</v>
-      </c>
-      <c r="C16" s="3" t="str">
-        <f t="shared" ref="C16:C22" si="0">DEC2HEX(HEX2DEC(C15)+HEX2DEC(F15))</f>
-        <v>2A000</v>
-      </c>
-      <c r="D16" s="3" t="str">
-        <f t="shared" ref="D16:D22" si="1">DEC2HEX(HEX2DEC($B$3)+HEX2DEC(C16))</f>
-        <v>802A000</v>
       </c>
       <c r="E16" s="3" t="str">
         <f>DEC2HEX(HEX2DEC(D16)+HEX2DEC(F16)-1)</f>
-        <v>803BFFF</v>
+        <v>8029FFF</v>
       </c>
       <c r="F16" s="8">
-        <f>F15</f>
         <v>12000</v>
       </c>
       <c r="G16" s="3">
@@ -983,38 +984,38 @@
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="B17" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B17" s="3">
+        <v>2</v>
+      </c>
+      <c r="C17" s="3" t="str">
+        <f t="shared" ref="C17:C22" si="0">DEC2HEX(HEX2DEC(C16)+HEX2DEC(F16))</f>
+        <v>2A000</v>
+      </c>
+      <c r="D17" s="3" t="str">
+        <f t="shared" ref="D17:D22" si="1">DEC2HEX(HEX2DEC($B$3)+HEX2DEC(C17))</f>
+        <v>802A000</v>
+      </c>
+      <c r="E17" s="3" t="str">
+        <f>DEC2HEX(HEX2DEC(D17)+HEX2DEC(F17)-1)</f>
+        <v>803BFFF</v>
+      </c>
+      <c r="F17" s="8">
+        <f>F16</f>
+        <v>12000</v>
+      </c>
+      <c r="G17" s="3">
+        <f>H17/1024</f>
+        <v>72</v>
+      </c>
+      <c r="H17" s="2">
+        <f>HEX2DEC(F17)</f>
+        <v>73728</v>
+      </c>
+      <c r="I17" s="13">
+        <f>H17/HEX2DEC($B$5)</f>
         <v>9</v>
-      </c>
-      <c r="C17" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v>3C000</v>
-      </c>
-      <c r="D17" s="3" t="str">
-        <f t="shared" si="1"/>
-        <v>803C000</v>
-      </c>
-      <c r="E17" s="3" t="str">
-        <f t="shared" ref="E17:E22" si="2">DEC2HEX(HEX2DEC(D17)+HEX2DEC(F17)-1)</f>
-        <v>803BFFF</v>
-      </c>
-      <c r="F17" s="3">
-        <f>IF(($B$6="N"),IF($B$7="N",10000,0),0)</f>
-        <v>0</v>
-      </c>
-      <c r="G17" s="3">
-        <f t="shared" ref="G17:G25" si="3">H17/1024</f>
-        <v>0</v>
-      </c>
-      <c r="H17" s="2">
-        <f t="shared" ref="H17:H21" si="4">HEX2DEC(F17)</f>
-        <v>0</v>
-      </c>
-      <c r="I17" s="13">
-        <f t="shared" ref="I17:I21" si="5">H17/HEX2DEC($B$5)</f>
-        <v>0</v>
       </c>
       <c r="J17" s="13" t="s">
         <v>6</v>
@@ -1026,10 +1027,10 @@
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B18" s="3">
-        <v>4</v>
+        <v>8</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="C18" s="3" t="str">
         <f t="shared" si="0"/>
@@ -1040,23 +1041,23 @@
         <v>803C000</v>
       </c>
       <c r="E18" s="3" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="E18:E22" si="2">DEC2HEX(HEX2DEC(D18)+HEX2DEC(F18)-1)</f>
         <v>803BFFF</v>
       </c>
       <c r="F18" s="3">
-        <f>$B$11</f>
+        <f>IF(($B$6="N"),IF($B$7="N",10000,0),0)</f>
         <v>0</v>
       </c>
       <c r="G18" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="G18:G25" si="3">H18/1024</f>
         <v>0</v>
       </c>
       <c r="H18" s="2">
-        <f t="shared" si="4"/>
+        <f t="shared" ref="H18:H22" si="4">HEX2DEC(F18)</f>
         <v>0</v>
       </c>
       <c r="I18" s="13">
-        <f t="shared" si="5"/>
+        <f t="shared" ref="I18:I22" si="5">H18/HEX2DEC($B$5)</f>
         <v>0</v>
       </c>
       <c r="J18" s="13" t="s">
@@ -1069,10 +1070,10 @@
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="B19" s="3">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C19" s="3" t="str">
         <f t="shared" si="0"/>
@@ -1084,23 +1085,23 @@
       </c>
       <c r="E19" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>8119FFF</v>
-      </c>
-      <c r="F19" s="14" t="str">
-        <f>DEC2HEX(IF($B$6="N",ROUNDDOWN((HEX2DEC(B4)-HEX2DEC(F14)-HEX2DEC(F15)-HEX2DEC(F16)-HEX2DEC(F17)-HEX2DEC(F22)-HEX2DEC(F18)-HEX2DEC(F21))/2/HEX2DEC($B$5),0)*HEX2DEC($B$5),(HEX2DEC(B4)-HEX2DEC(F14)-HEX2DEC(F15)-HEX2DEC(F16)-HEX2DEC(F17)-HEX2DEC(F22)-HEX2DEC(F18)-HEX2DEC(F21))))</f>
-        <v>DE000</v>
+        <v>803BFFF</v>
+      </c>
+      <c r="F19" s="3">
+        <f>$B$11</f>
+        <v>0</v>
       </c>
       <c r="G19" s="3">
         <f t="shared" si="3"/>
-        <v>888</v>
+        <v>0</v>
       </c>
       <c r="H19" s="2">
         <f t="shared" si="4"/>
-        <v>909312</v>
+        <v>0</v>
       </c>
       <c r="I19" s="13">
         <f t="shared" si="5"/>
-        <v>111</v>
+        <v>0</v>
       </c>
       <c r="J19" s="13" t="s">
         <v>6</v>
@@ -1112,25 +1113,25 @@
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B20" s="3">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C20" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>11A000</v>
+        <v>3C000</v>
       </c>
       <c r="D20" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>811A000</v>
+        <v>803C000</v>
       </c>
       <c r="E20" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>81F7FFF</v>
+        <v>8119FFF</v>
       </c>
       <c r="F20" s="14" t="str">
-        <f>IF($B$6="N",F19,0)</f>
+        <f>DEC2HEX(IF($B$6="N",ROUNDDOWN((HEX2DEC(B4)-HEX2DEC(F14)-HEX2DEC(F16)-HEX2DEC(F17)-HEX2DEC(F18)-HEX2DEC(F15)-HEX2DEC(F19)-HEX2DEC(F22))/2/HEX2DEC($B$5),0)*HEX2DEC($B$5),(HEX2DEC(B4)-HEX2DEC(F14)-HEX2DEC(F16)-HEX2DEC(F17)-HEX2DEC(F18)-HEX2DEC(F15)-HEX2DEC(F19)-HEX2DEC(F22))))</f>
         <v>DE000</v>
       </c>
       <c r="G20" s="3">
@@ -1155,38 +1156,38 @@
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="B21" s="3">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C21" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>1F8000</v>
+        <v>11A000</v>
       </c>
       <c r="D21" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>81F8000</v>
+        <v>811A000</v>
       </c>
       <c r="E21" s="3" t="str">
         <f t="shared" si="2"/>
         <v>81F7FFF</v>
       </c>
-      <c r="F21" s="3">
-        <f>IF($B$10="Y",F18,0)</f>
-        <v>0</v>
+      <c r="F21" s="14" t="str">
+        <f>IF($B$6="N",F20,0)</f>
+        <v>DE000</v>
       </c>
       <c r="G21" s="3">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>888</v>
       </c>
       <c r="H21" s="2">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>909312</v>
       </c>
       <c r="I21" s="13">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>111</v>
       </c>
       <c r="J21" s="13" t="s">
         <v>6</v>
@@ -1198,10 +1199,10 @@
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>10</v>
+        <v>13</v>
+      </c>
+      <c r="B22" s="3">
+        <v>6</v>
       </c>
       <c r="C22" s="3" t="str">
         <f t="shared" si="0"/>
@@ -1213,26 +1214,26 @@
       </c>
       <c r="E22" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>81FFFFF</v>
-      </c>
-      <c r="F22" s="8">
-        <f>$B$9</f>
-        <v>8000</v>
+        <v>81F7FFF</v>
+      </c>
+      <c r="F22" s="3">
+        <f>IF($B$10="Y",F19,0)</f>
+        <v>0</v>
       </c>
       <c r="G22" s="3">
-        <f>H22/1024</f>
-        <v>32</v>
+        <f t="shared" si="3"/>
+        <v>0</v>
       </c>
       <c r="H22" s="2">
-        <f>HEX2DEC(F22)</f>
-        <v>32768</v>
+        <f t="shared" si="4"/>
+        <v>0</v>
       </c>
       <c r="I22" s="13">
-        <f>H22/HEX2DEC($B$5)</f>
-        <v>4</v>
+        <f t="shared" si="5"/>
+        <v>0</v>
       </c>
       <c r="J22" s="13" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="K22" s="13" t="s">
         <v>6</v>
@@ -1241,7 +1242,7 @@
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
@@ -1249,27 +1250,27 @@
       <c r="E23" s="1"/>
       <c r="F23" s="10" t="str">
         <f>DEC2HEX(H23)</f>
-        <v>200000</v>
+        <v>1FE000</v>
       </c>
       <c r="G23" s="1">
         <f t="shared" si="3"/>
-        <v>2048</v>
+        <v>2040</v>
       </c>
       <c r="H23" s="11">
         <f>SUM(H14:H22)</f>
-        <v>2097152</v>
+        <v>2088960</v>
       </c>
       <c r="I23">
         <f>H23/HEX2DEC($B$5)</f>
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" s="9" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B24" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F24" s="11">
         <f>$B$4</f>
@@ -1290,28 +1291,36 @@
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="9" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F25" s="11" t="str">
         <f>DEC2HEX(H25)</f>
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="G25" s="1">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="H25" s="11">
         <f>H24-H23</f>
-        <v>0</v>
+        <v>8192</v>
       </c>
       <c r="I25">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A27" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="B27">
+        <v>16000</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" s="12" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B28" s="7" t="s">
         <v>3</v>
@@ -1323,30 +1332,30 @@
         <v>1</v>
       </c>
       <c r="E28" s="7" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G28" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="H28" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="I28" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="J28" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="H28" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="I28" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="J28" s="12" t="s">
-        <v>28</v>
-      </c>
       <c r="K28" s="12" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" s="8" t="s">
-        <v>2</v>
+        <v>36</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>2</v>
@@ -1359,8 +1368,8 @@
         <v>8000000</v>
       </c>
       <c r="E29" s="3" t="str">
-        <f>DEC2HEX(HEX2DEC(D29)+HEX2DEC(F29)-1)</f>
-        <v>8017FFF</v>
+        <f>DEC2HEX(HEX2DEC(D29)+IF(($B$8="Y"),HEX2DEC(F29)-HEX2DEC(F30),HEX2DEC(F29))-1)</f>
+        <v>8011FFF</v>
       </c>
       <c r="F29" s="8">
         <v>18000</v>
@@ -1386,55 +1395,55 @@
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" s="8" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C30" s="3" t="str">
-        <f>DEC2HEX(HEX2DEC(C29)+HEX2DEC(F29))</f>
-        <v>18000</v>
+        <f>DEC2HEX(HEX2DEC(C29)+HEX2DEC(F29)-HEX2DEC(F30))</f>
+        <v>12000</v>
       </c>
       <c r="D30" s="3" t="str">
         <f>DEC2HEX(HEX2DEC($B$3)+HEX2DEC(C30))</f>
-        <v>8018000</v>
+        <v>8012000</v>
       </c>
       <c r="E30" s="3" t="str">
-        <f t="shared" ref="E30:E35" si="7">DEC2HEX(HEX2DEC(D30)+HEX2DEC(F30)-1)</f>
+        <f>DEC2HEX(HEX2DEC(D30)+HEX2DEC(F30)-1)</f>
         <v>8017FFF</v>
       </c>
-      <c r="F30" s="3">
-        <f>IF(($B$6="N"),IF($B$7="N",10000,0),0)</f>
-        <v>0</v>
+      <c r="F30" s="8">
+        <f>$B$9</f>
+        <v>6000</v>
       </c>
       <c r="G30" s="3">
-        <f t="shared" ref="G30:G38" si="8">H30/1024</f>
-        <v>0</v>
+        <f>H30/1024</f>
+        <v>24</v>
       </c>
       <c r="H30" s="2">
-        <f t="shared" ref="H30:H34" si="9">HEX2DEC(F30)</f>
-        <v>0</v>
+        <f>HEX2DEC(F30)</f>
+        <v>24576</v>
       </c>
       <c r="I30" s="13">
-        <f t="shared" ref="I30:I34" si="10">H30/HEX2DEC($B$5)</f>
-        <v>0</v>
+        <f>H30/HEX2DEC($B$5)</f>
+        <v>3</v>
       </c>
       <c r="J30" s="13" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="K30" s="13" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" s="8" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="B31" s="3">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C31" s="3" t="str">
-        <f>DEC2HEX(HEX2DEC(C30)+HEX2DEC(F30))</f>
+        <f>DEC2HEX(HEX2DEC(C29)+HEX2DEC(F29))</f>
         <v>18000</v>
       </c>
       <c r="D31" s="3" t="str">
@@ -1442,24 +1451,23 @@
         <v>8018000</v>
       </c>
       <c r="E31" s="3" t="str">
-        <f t="shared" si="7"/>
-        <v>8017FFF</v>
-      </c>
-      <c r="F31" s="3">
-        <f>$B$11</f>
-        <v>0</v>
+        <f>DEC2HEX(HEX2DEC(D31)+HEX2DEC(F31)-1)</f>
+        <v>8029FFF</v>
+      </c>
+      <c r="F31" s="8">
+        <v>12000</v>
       </c>
       <c r="G31" s="3">
-        <f t="shared" si="8"/>
-        <v>0</v>
+        <f>H31/1024</f>
+        <v>72</v>
       </c>
       <c r="H31" s="2">
-        <f t="shared" si="9"/>
-        <v>0</v>
+        <f>HEX2DEC(F31)</f>
+        <v>73728</v>
       </c>
       <c r="I31" s="13">
-        <f t="shared" si="10"/>
-        <v>0</v>
+        <f>H31/HEX2DEC($B$5)</f>
+        <v>9</v>
       </c>
       <c r="J31" s="13" t="s">
         <v>6</v>
@@ -1470,37 +1478,38 @@
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" s="8" t="s">
-        <v>12</v>
+        <v>38</v>
       </c>
       <c r="B32" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C32" s="3" t="str">
-        <f t="shared" ref="C32:C34" si="11">DEC2HEX(HEX2DEC(C31)+HEX2DEC(F31))</f>
-        <v>18000</v>
+        <f t="shared" ref="C32:C37" si="7">DEC2HEX(HEX2DEC(C31)+HEX2DEC(F31))</f>
+        <v>2A000</v>
       </c>
       <c r="D32" s="3" t="str">
-        <f t="shared" ref="D32:D34" si="12">DEC2HEX(HEX2DEC($B$3)+HEX2DEC(C32))</f>
-        <v>8018000</v>
+        <f t="shared" ref="D32:D37" si="8">DEC2HEX(HEX2DEC($B$3)+HEX2DEC(C32))</f>
+        <v>802A000</v>
       </c>
       <c r="E32" s="3" t="str">
-        <f t="shared" si="7"/>
-        <v>802DFFF</v>
-      </c>
-      <c r="F32" s="15">
-        <v>16000</v>
+        <f>DEC2HEX(HEX2DEC(D32)+HEX2DEC(F32)-1)</f>
+        <v>803BFFF</v>
+      </c>
+      <c r="F32" s="8">
+        <f>F31</f>
+        <v>12000</v>
       </c>
       <c r="G32" s="3">
-        <f t="shared" si="8"/>
-        <v>88</v>
+        <f>H32/1024</f>
+        <v>72</v>
       </c>
       <c r="H32" s="2">
-        <f t="shared" si="9"/>
-        <v>90112</v>
+        <f>HEX2DEC(F32)</f>
+        <v>73728</v>
       </c>
       <c r="I32" s="13">
-        <f t="shared" si="10"/>
-        <v>11</v>
+        <f>H32/HEX2DEC($B$5)</f>
+        <v>9</v>
       </c>
       <c r="J32" s="13" t="s">
         <v>6</v>
@@ -1511,38 +1520,38 @@
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="B33" s="3">
-        <v>2</v>
+        <v>8</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="C33" s="3" t="str">
-        <f t="shared" si="11"/>
-        <v>2E000</v>
+        <f t="shared" si="7"/>
+        <v>3C000</v>
       </c>
       <c r="D33" s="3" t="str">
-        <f t="shared" si="12"/>
-        <v>802E000</v>
+        <f t="shared" si="8"/>
+        <v>803C000</v>
       </c>
       <c r="E33" s="3" t="str">
-        <f t="shared" si="7"/>
-        <v>8043FFF</v>
-      </c>
-      <c r="F33" s="15">
-        <f>IF($B$6="N",F32,0)</f>
-        <v>16000</v>
+        <f t="shared" ref="E33:E37" si="9">DEC2HEX(HEX2DEC(D33)+HEX2DEC(F33)-1)</f>
+        <v>803BFFF</v>
+      </c>
+      <c r="F33" s="3">
+        <f>IF(($B$6="N"),IF($B$7="N",10000,0),0)</f>
+        <v>0</v>
       </c>
       <c r="G33" s="3">
-        <f t="shared" si="8"/>
-        <v>88</v>
+        <f t="shared" ref="G33:G40" si="10">H33/1024</f>
+        <v>0</v>
       </c>
       <c r="H33" s="2">
-        <f t="shared" si="9"/>
-        <v>90112</v>
+        <f t="shared" ref="H33:H37" si="11">HEX2DEC(F33)</f>
+        <v>0</v>
       </c>
       <c r="I33" s="13">
-        <f t="shared" si="10"/>
-        <v>11</v>
+        <f t="shared" ref="I33:I37" si="12">H33/HEX2DEC($B$5)</f>
+        <v>0</v>
       </c>
       <c r="J33" s="13" t="s">
         <v>6</v>
@@ -1553,37 +1562,37 @@
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" s="8" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B34" s="3">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C34" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>3C000</v>
+      </c>
+      <c r="D34" s="3" t="str">
+        <f t="shared" si="8"/>
+        <v>803C000</v>
+      </c>
+      <c r="E34" s="3" t="str">
+        <f t="shared" si="9"/>
+        <v>803BFFF</v>
+      </c>
+      <c r="F34" s="3">
+        <f>$B$11</f>
+        <v>0</v>
+      </c>
+      <c r="G34" s="3">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="H34" s="2">
         <f t="shared" si="11"/>
-        <v>44000</v>
-      </c>
-      <c r="D34" s="3" t="str">
+        <v>0</v>
+      </c>
+      <c r="I34" s="13">
         <f t="shared" si="12"/>
-        <v>8044000</v>
-      </c>
-      <c r="E34" s="3" t="str">
-        <f t="shared" si="7"/>
-        <v>8043FFF</v>
-      </c>
-      <c r="F34" s="3">
-        <f>IF($B$10="Y",F31,0)</f>
-        <v>0</v>
-      </c>
-      <c r="G34" s="3">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="H34" s="2">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="I34" s="13">
-        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="J34" s="13" t="s">
@@ -1595,146 +1604,230 @@
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B35" s="3" t="s">
-        <v>10</v>
+        <v>34</v>
+      </c>
+      <c r="B35" s="3">
+        <v>0</v>
       </c>
       <c r="C35" s="3" t="str">
-        <f>DEC2HEX(HEX2DEC(C34)+HEX2DEC(F34))</f>
-        <v>44000</v>
+        <f t="shared" si="7"/>
+        <v>3C000</v>
       </c>
       <c r="D35" s="3" t="str">
-        <f>DEC2HEX(HEX2DEC($B$3)+HEX2DEC(C35))</f>
-        <v>8044000</v>
+        <f t="shared" si="8"/>
+        <v>803C000</v>
       </c>
       <c r="E35" s="3" t="str">
+        <f t="shared" si="9"/>
+        <v>8051FFF</v>
+      </c>
+      <c r="F35" s="15">
+        <f>B27</f>
+        <v>16000</v>
+      </c>
+      <c r="G35" s="3">
+        <f t="shared" si="10"/>
+        <v>88</v>
+      </c>
+      <c r="H35" s="2">
+        <f t="shared" si="11"/>
+        <v>90112</v>
+      </c>
+      <c r="I35" s="13">
+        <f t="shared" si="12"/>
+        <v>11</v>
+      </c>
+      <c r="J35" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="K35" s="13" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A36" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="B36" s="3">
+        <v>2</v>
+      </c>
+      <c r="C36" s="3" t="str">
         <f t="shared" si="7"/>
-        <v>804BFFF</v>
-      </c>
-      <c r="F35" s="8">
-        <f>$B$9</f>
-        <v>8000</v>
-      </c>
-      <c r="G35" s="3">
-        <f>H35/1024</f>
-        <v>32</v>
-      </c>
-      <c r="H35" s="2">
-        <f>HEX2DEC(F35)</f>
-        <v>32768</v>
-      </c>
-      <c r="I35" s="13">
-        <f>H35/HEX2DEC($B$5)</f>
-        <v>4</v>
-      </c>
-      <c r="J35" s="13" t="s">
+        <v>52000</v>
+      </c>
+      <c r="D36" s="3" t="str">
+        <f t="shared" si="8"/>
+        <v>8052000</v>
+      </c>
+      <c r="E36" s="3" t="str">
+        <f t="shared" si="9"/>
+        <v>8067FFF</v>
+      </c>
+      <c r="F36" s="15">
+        <f>IF($B$6="N",F35,0)</f>
+        <v>16000</v>
+      </c>
+      <c r="G36" s="3">
+        <f t="shared" si="10"/>
+        <v>88</v>
+      </c>
+      <c r="H36" s="2">
+        <f t="shared" si="11"/>
+        <v>90112</v>
+      </c>
+      <c r="I36" s="13">
+        <f t="shared" si="12"/>
         <v>11</v>
       </c>
-      <c r="K35" s="13" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A36" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B36" s="1"/>
-      <c r="C36" s="1"/>
-      <c r="D36" s="1"/>
-      <c r="E36" s="1"/>
-      <c r="F36" s="10" t="str">
-        <f>DEC2HEX(H36)</f>
-        <v>4C000</v>
-      </c>
-      <c r="G36" s="1">
+      <c r="J36" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="K36" s="13" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A37" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B37" s="3">
+        <v>6</v>
+      </c>
+      <c r="C37" s="3" t="str">
+        <f t="shared" si="7"/>
+        <v>68000</v>
+      </c>
+      <c r="D37" s="3" t="str">
         <f t="shared" si="8"/>
-        <v>304</v>
-      </c>
-      <c r="H36" s="11">
-        <f>SUM(H29:H35)</f>
-        <v>311296</v>
-      </c>
-      <c r="I36">
-        <f>H36/HEX2DEC($B$5)</f>
-        <v>38</v>
-      </c>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A37" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="B37" t="s">
-        <v>21</v>
-      </c>
-      <c r="F37" s="11">
+        <v>8068000</v>
+      </c>
+      <c r="E37" s="3" t="str">
+        <f t="shared" si="9"/>
+        <v>8067FFF</v>
+      </c>
+      <c r="F37" s="3">
+        <f>IF($B$10="Y",F34,0)</f>
+        <v>0</v>
+      </c>
+      <c r="G37" s="3">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="H37" s="2">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="I37" s="13">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="J37" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="K37" s="13" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A38" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B38" s="1"/>
+      <c r="C38" s="1"/>
+      <c r="D38" s="1"/>
+      <c r="E38" s="1"/>
+      <c r="F38" s="10" t="str">
+        <f>DEC2HEX(H38)</f>
+        <v>6E000</v>
+      </c>
+      <c r="G38" s="1">
+        <f t="shared" si="10"/>
+        <v>440</v>
+      </c>
+      <c r="H38" s="11">
+        <f>SUM(H29:H37)</f>
+        <v>450560</v>
+      </c>
+      <c r="I38">
+        <f>H38/HEX2DEC($B$5)</f>
+        <v>55</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A39" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B39" t="s">
+        <v>19</v>
+      </c>
+      <c r="F39" s="11">
         <f>$B$4</f>
         <v>200000</v>
       </c>
-      <c r="G37" s="1">
-        <f t="shared" si="8"/>
+      <c r="G39" s="1">
+        <f t="shared" si="10"/>
         <v>2048</v>
       </c>
-      <c r="H37" s="11">
-        <f>HEX2DEC(F37)</f>
+      <c r="H39" s="11">
+        <f>HEX2DEC(F39)</f>
         <v>2097152</v>
       </c>
-      <c r="I37">
-        <f t="shared" ref="I37:I38" si="13">H37/HEX2DEC($B$5)</f>
+      <c r="I39">
+        <f t="shared" ref="I39:I40" si="13">H39/HEX2DEC($B$5)</f>
         <v>256</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A38" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="F38" s="11" t="str">
-        <f>DEC2HEX(H38)</f>
-        <v>1B4000</v>
-      </c>
-      <c r="G38" s="1">
-        <f t="shared" si="8"/>
-        <v>1744</v>
-      </c>
-      <c r="H38" s="11">
-        <f>H37-H36</f>
-        <v>1785856</v>
-      </c>
-      <c r="I38">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A40" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="F40" s="11" t="str">
+        <f>DEC2HEX(H40)</f>
+        <v>192000</v>
+      </c>
+      <c r="G40" s="1">
+        <f t="shared" si="10"/>
+        <v>1608</v>
+      </c>
+      <c r="H40" s="11">
+        <f>H39-H38</f>
+        <v>1646592</v>
+      </c>
+      <c r="I40">
         <f t="shared" si="13"/>
-        <v>218</v>
+        <v>201</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="B6:B8 B10">
-    <cfRule type="cellIs" dxfId="5" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="7" operator="equal">
       <formula>"Y"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="4" priority="8" operator="equal">
       <formula>"N"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J29:K35">
-    <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
+  <conditionalFormatting sqref="J14:L22">
+    <cfRule type="cellIs" dxfId="3" priority="5" operator="equal">
       <formula>"N"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="6" operator="equal">
       <formula>"Y"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J14:L22">
-    <cfRule type="cellIs" dxfId="1" priority="3" operator="equal">
+  <conditionalFormatting sqref="J29:K37">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>"N"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
       <formula>"Y"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B6:B8 B10 J14:L22 J29:K35" xr:uid="{EBA8029F-00D4-49E4-8B84-75C1EA9F44E8}">
+  <dataValidations disablePrompts="1" count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B6:B8 B10 J14:L22 J29:K37" xr:uid="{EBA8029F-00D4-49E4-8B84-75C1EA9F44E8}">
       <formula1>$B$1:$B$2</formula1>
     </dataValidation>
-    <dataValidation type="decimal" operator="lessThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Error" error="Total size consumed cannot exceed total user flash size!" sqref="H23 H36" xr:uid="{1D140836-F0E9-4E03-84AE-026A1CDC9976}">
+    <dataValidation type="decimal" operator="lessThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Error" error="Total size consumed cannot exceed total user flash size!" sqref="H23 H38" xr:uid="{1D140836-F0E9-4E03-84AE-026A1CDC9976}">
       <formula1>H24</formula1>
     </dataValidation>
   </dataValidations>
@@ -1743,6 +1836,18 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5FFBD9D-4558-48E5-B9F3-C9C695119802}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.140625" customWidth="1"/>
+  </cols>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{cf8c7287-838c-46dd-b281-b1140229e67a}" enabled="1" method="Privileged" siteId="{75e027c9-20d5-47d5-b82f-77d7cd041e8f}" contentBits="0" removed="0"/>

</xml_diff>

<commit_message>
[ROT] Test Overwrite mode wo/ standalone loader for IAR and CubeIDE
</commit_message>
<xml_diff>
--- a/Projects/NUCLEO-H563ZI/ROT_Provisioning/OEMiROT_OEMuROT/OEMiROT_OEMuROT_flash_layout.xlsx
+++ b/Projects/NUCLEO-H563ZI/ROT_Provisioning/OEMiROT_OEMuROT/OEMiROT_OEMuROT_flash_layout.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ST\Cube\Cube1\STM32CubeH5\Projects\NUCLEO-H563ZI\ROT_Provisioning\OEMiROT_OEMuROT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D136FC5F-D23C-4402-B307-40ECB6629AA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{685360A6-D1AB-41FA-8518-E1D6A05E02AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{973ADE99-8809-4282-875C-44A8EA15E93C}"/>
+    <workbookView xWindow="-165" yWindow="-165" windowWidth="29130" windowHeight="15810" tabRatio="594" xr2:uid="{973ADE99-8809-4282-875C-44A8EA15E93C}"/>
   </bookViews>
   <sheets>
     <sheet name="OEMiROT+OEMuROT Flash Layout" sheetId="1" r:id="rId1"/>
@@ -1243,22 +1243,22 @@
       </c>
       <c r="E19" s="3" t="str">
         <f>DEC2HEX(HEX2DEC(D19)+HEX2DEC(F19)-1)</f>
-        <v>8039FFF</v>
+        <v>803FFFF</v>
       </c>
       <c r="F19" s="8">
-        <v>12000</v>
+        <v>18000</v>
       </c>
       <c r="G19" s="3">
         <f>H19/1024</f>
-        <v>72</v>
+        <v>96</v>
       </c>
       <c r="H19" s="2">
         <f>HEX2DEC(F19)</f>
-        <v>73728</v>
+        <v>98304</v>
       </c>
       <c r="I19" s="13">
         <f>H19/HEX2DEC($B$5)</f>
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="J19" s="13" t="s">
         <v>5</v>
@@ -1277,31 +1277,31 @@
       </c>
       <c r="C20" s="3" t="str">
         <f t="shared" ref="C20:C25" si="1">DEC2HEX(HEX2DEC(C19)+HEX2DEC(F19))</f>
-        <v>3A000</v>
+        <v>40000</v>
       </c>
       <c r="D20" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>803A000</v>
+        <v>8040000</v>
       </c>
       <c r="E20" s="3" t="str">
         <f>DEC2HEX(HEX2DEC(D20)+HEX2DEC(F20)-1)</f>
-        <v>804BFFF</v>
+        <v>8057FFF</v>
       </c>
       <c r="F20" s="8">
         <f>F19</f>
-        <v>12000</v>
+        <v>18000</v>
       </c>
       <c r="G20" s="3">
         <f>H20/1024</f>
-        <v>72</v>
+        <v>96</v>
       </c>
       <c r="H20" s="2">
         <f>HEX2DEC(F20)</f>
-        <v>73728</v>
+        <v>98304</v>
       </c>
       <c r="I20" s="13">
         <f>H20/HEX2DEC($B$5)</f>
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="J20" s="13" t="s">
         <v>5</v>
@@ -1320,15 +1320,15 @@
       </c>
       <c r="C21" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>4C000</v>
+        <v>58000</v>
       </c>
       <c r="D21" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>804C000</v>
+        <v>8058000</v>
       </c>
       <c r="E21" s="3" t="str">
         <f>DEC2HEX(HEX2DEC(D21)+HEX2DEC(F21)-1)</f>
-        <v>805BFFF</v>
+        <v>8067FFF</v>
       </c>
       <c r="F21" s="3">
         <f>IF(($B$8="N"),IF($B$9="N",10000,0),0)</f>
@@ -1363,15 +1363,15 @@
       </c>
       <c r="C22" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>5C000</v>
+        <v>68000</v>
       </c>
       <c r="D22" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>805C000</v>
+        <v>8068000</v>
       </c>
       <c r="E22" s="3" t="str">
         <f t="shared" ref="E22:E25" si="2">DEC2HEX(HEX2DEC(D22)+HEX2DEC(F22)-1)</f>
-        <v>805BFFF</v>
+        <v>8067FFF</v>
       </c>
       <c r="F22" s="3">
         <f>$B$13</f>
@@ -1406,31 +1406,31 @@
       </c>
       <c r="C23" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>5C000</v>
+        <v>68000</v>
       </c>
       <c r="D23" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>805C000</v>
+        <v>8068000</v>
       </c>
       <c r="E23" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>8129FFF</v>
+        <v>812FFFF</v>
       </c>
       <c r="F23" s="14" t="str">
         <f>DEC2HEX(IF($B$6="N",ROUNDDOWN((HEX2DEC(B4)-HEX2DEC(F16)-HEX2DEC(F19)-HEX2DEC(F20)-HEX2DEC(F18)-HEX2DEC(F21)-HEX2DEC(F17)-HEX2DEC(F22)-HEX2DEC(F25))/2/HEX2DEC($B$5),0)*HEX2DEC($B$5),(HEX2DEC(B4)-HEX2DEC(F16)-HEX2DEC(F19)-HEX2DEC(F20)-HEX2DEC(F18)-HEX2DEC(F21)-HEX2DEC(F17)-HEX2DEC(F22)-HEX2DEC(F25))))</f>
-        <v>CE000</v>
+        <v>C8000</v>
       </c>
       <c r="G23" s="3">
         <f t="shared" si="3"/>
-        <v>824</v>
+        <v>800</v>
       </c>
       <c r="H23" s="2">
         <f t="shared" si="4"/>
-        <v>843776</v>
+        <v>819200</v>
       </c>
       <c r="I23" s="13">
         <f t="shared" si="5"/>
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="J23" s="13" t="s">
         <v>5</v>
@@ -1449,11 +1449,11 @@
       </c>
       <c r="C24" s="3" t="str">
         <f t="shared" si="1"/>
-        <v>12A000</v>
+        <v>130000</v>
       </c>
       <c r="D24" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>812A000</v>
+        <v>8130000</v>
       </c>
       <c r="E24" s="3" t="str">
         <f t="shared" si="2"/>
@@ -1461,19 +1461,19 @@
       </c>
       <c r="F24" s="14" t="str">
         <f>IF($B$6="N",F23,0)</f>
-        <v>CE000</v>
+        <v>C8000</v>
       </c>
       <c r="G24" s="3">
         <f t="shared" si="3"/>
-        <v>824</v>
+        <v>800</v>
       </c>
       <c r="H24" s="2">
         <f t="shared" si="4"/>
-        <v>843776</v>
+        <v>819200</v>
       </c>
       <c r="I24" s="13">
         <f t="shared" si="5"/>
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="J24" s="13" t="s">
         <v>5</v>

</xml_diff>